<commit_message>
actualizo con analisis x audios
</commit_message>
<xml_diff>
--- a/outputs/classification_report_nsb_nsm_con_tiempo.xlsx
+++ b/outputs/classification_report_nsb_nsm_con_tiempo.xlsx
@@ -463,19 +463,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40.4</v>
+        <v>52.8</v>
       </c>
       <c r="C2" t="n">
-        <v>72</v>
+        <v>70.8</v>
       </c>
       <c r="D2" t="n">
-        <v>51.8</v>
+        <v>60.4</v>
       </c>
       <c r="E2" t="n">
-        <v>229744</v>
+        <v>147933</v>
       </c>
       <c r="F2" t="n">
-        <v>38.29</v>
+        <v>24.66</v>
       </c>
     </row>
     <row r="3">
@@ -485,19 +485,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30.3</v>
+        <v>43.4</v>
       </c>
       <c r="C3" t="n">
-        <v>45.3</v>
+        <v>42.5</v>
       </c>
       <c r="D3" t="n">
-        <v>36.3</v>
+        <v>42.9</v>
       </c>
       <c r="E3" t="n">
-        <v>240470</v>
+        <v>165400</v>
       </c>
       <c r="F3" t="n">
-        <v>40.08</v>
+        <v>27.57</v>
       </c>
     </row>
     <row r="4">
@@ -507,19 +507,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38.4</v>
+        <v>52.4</v>
       </c>
       <c r="C4" t="n">
-        <v>56.3</v>
+        <v>52.4</v>
       </c>
       <c r="D4" t="n">
-        <v>45.6</v>
+        <v>52.4</v>
       </c>
       <c r="E4" t="n">
-        <v>390196</v>
+        <v>318769</v>
       </c>
       <c r="F4" t="n">
-        <v>65.03</v>
+        <v>53.13</v>
       </c>
     </row>
     <row r="5">
@@ -529,19 +529,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32.7</v>
+        <v>40.1</v>
       </c>
       <c r="C5" t="n">
-        <v>40.6</v>
+        <v>32</v>
       </c>
       <c r="D5" t="n">
-        <v>36.2</v>
+        <v>35.6</v>
       </c>
       <c r="E5" t="n">
-        <v>142584</v>
+        <v>115518</v>
       </c>
       <c r="F5" t="n">
-        <v>23.76</v>
+        <v>19.25</v>
       </c>
     </row>
     <row r="6">
@@ -551,19 +551,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.59999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>57.2</v>
+        <v>73.8</v>
       </c>
       <c r="D6" t="n">
-        <v>69.2</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>1857437</v>
+        <v>951762</v>
       </c>
       <c r="F6" t="n">
-        <v>309.57</v>
+        <v>158.63</v>
       </c>
     </row>
     <row r="7">
@@ -573,19 +573,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>75.7</v>
+        <v>71.8</v>
       </c>
       <c r="D7" t="n">
-        <v>61.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>902563</v>
+        <v>668238</v>
       </c>
       <c r="F7" t="n">
-        <v>150.43</v>
+        <v>111.37</v>
       </c>
     </row>
     <row r="8">
@@ -595,19 +595,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>56.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>61.1</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>58.9</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>3762994</v>
+        <v>2367620</v>
       </c>
       <c r="F8" t="n">
-        <v>627.17</v>
+        <v>394.6</v>
       </c>
     </row>
     <row r="9">
@@ -617,19 +617,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>46.9</v>
+        <v>57.3</v>
       </c>
       <c r="C9" t="n">
-        <v>57.9</v>
+        <v>57.2</v>
       </c>
       <c r="D9" t="n">
-        <v>50.1</v>
+        <v>56.9</v>
       </c>
       <c r="E9" t="n">
-        <v>3762994</v>
+        <v>2367620</v>
       </c>
       <c r="F9" t="n">
-        <v>627.17</v>
+        <v>394.6</v>
       </c>
     </row>
     <row r="10">
@@ -639,19 +639,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>65.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>61.1</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>60.5</v>
+        <v>67.3</v>
       </c>
       <c r="E10" t="n">
-        <v>3762994</v>
+        <v>2367620</v>
       </c>
       <c r="F10" t="n">
-        <v>627.17</v>
+        <v>394.6</v>
       </c>
     </row>
     <row r="11">
@@ -661,19 +661,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>58.4</v>
+        <v>67.2</v>
       </c>
       <c r="C11" t="n">
-        <v>59.8</v>
+        <v>68.5</v>
       </c>
       <c r="D11" t="n">
-        <v>58.7</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>3762994</v>
+        <v>2367620</v>
       </c>
       <c r="F11" t="n">
-        <v>627.17</v>
+        <v>394.6</v>
       </c>
     </row>
   </sheetData>
@@ -724,19 +724,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="C2" t="n">
-        <v>54.3</v>
+        <v>75.7</v>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>262539</v>
+        <v>185345</v>
       </c>
       <c r="F2" t="n">
-        <v>43.76</v>
+        <v>30.89</v>
       </c>
     </row>
     <row r="3">
@@ -746,19 +746,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="n">
-        <v>18.6</v>
+        <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>19.7</v>
+        <v>24.8</v>
       </c>
       <c r="E3" t="n">
-        <v>119930</v>
+        <v>82713</v>
       </c>
       <c r="F3" t="n">
-        <v>19.99</v>
+        <v>13.79</v>
       </c>
     </row>
     <row r="4">
@@ -768,19 +768,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="C4" t="n">
-        <v>59.9</v>
+        <v>72.7</v>
       </c>
       <c r="D4" t="n">
-        <v>55.1</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>400773</v>
+        <v>299118</v>
       </c>
       <c r="F4" t="n">
-        <v>66.8</v>
+        <v>49.85</v>
       </c>
     </row>
     <row r="5">
@@ -790,19 +790,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48.3</v>
+        <v>52.3</v>
       </c>
       <c r="C5" t="n">
-        <v>39.1</v>
+        <v>44.1</v>
       </c>
       <c r="D5" t="n">
-        <v>43.3</v>
+        <v>47.8</v>
       </c>
       <c r="E5" t="n">
-        <v>150885</v>
+        <v>133697</v>
       </c>
       <c r="F5" t="n">
-        <v>25.15</v>
+        <v>22.28</v>
       </c>
     </row>
     <row r="6">
@@ -812,19 +812,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>82.90000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>77.8</v>
+        <v>81.7</v>
       </c>
       <c r="D6" t="n">
-        <v>80.3</v>
+        <v>86.3</v>
       </c>
       <c r="E6" t="n">
-        <v>1495560</v>
+        <v>1150992</v>
       </c>
       <c r="F6" t="n">
-        <v>249.26</v>
+        <v>191.83</v>
       </c>
     </row>
     <row r="7">
@@ -834,19 +834,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>66.09999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>66.5</v>
+        <v>78.2</v>
       </c>
       <c r="E7" t="n">
-        <v>832442</v>
+        <v>637010</v>
       </c>
       <c r="F7" t="n">
-        <v>138.74</v>
+        <v>106.17</v>
       </c>
     </row>
     <row r="8">
@@ -856,19 +856,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69.2</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>66.8</v>
+        <v>76</v>
       </c>
       <c r="D8" t="n">
-        <v>68</v>
+        <v>76.5</v>
       </c>
       <c r="E8" t="n">
-        <v>3262129</v>
+        <v>2488875</v>
       </c>
       <c r="F8" t="n">
-        <v>543.6900000000001</v>
+        <v>414.81</v>
       </c>
     </row>
     <row r="9">
@@ -878,19 +878,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>55.8</v>
+        <v>62.6</v>
       </c>
       <c r="C9" t="n">
-        <v>52.6</v>
+        <v>63.6</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>62.9</v>
       </c>
       <c r="E9" t="n">
-        <v>3262129</v>
+        <v>2488875</v>
       </c>
       <c r="F9" t="n">
-        <v>543.6900000000001</v>
+        <v>414.81</v>
       </c>
     </row>
     <row r="10">
@@ -900,19 +900,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>69.5</v>
+        <v>78.2</v>
       </c>
       <c r="C10" t="n">
-        <v>66.8</v>
+        <v>76</v>
       </c>
       <c r="D10" t="n">
-        <v>68</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>3262129</v>
+        <v>2488875</v>
       </c>
       <c r="F10" t="n">
-        <v>543.6900000000001</v>
+        <v>414.81</v>
       </c>
     </row>
     <row r="11">
@@ -922,19 +922,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C11" t="n">
-        <v>70.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>70.2</v>
+        <v>77.2</v>
       </c>
       <c r="E11" t="n">
-        <v>3262129</v>
+        <v>2488875</v>
       </c>
       <c r="F11" t="n">
-        <v>543.6900000000001</v>
+        <v>414.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>